<commit_message>
Initial AI Recruitment Platform
</commit_message>
<xml_diff>
--- a/reports/candidates.xlsx
+++ b/reports/candidates.xlsx
@@ -455,7 +455,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -488,7 +488,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>

</xml_diff>